<commit_message>
Add SQL analysis queries
</commit_message>
<xml_diff>
--- a/data/raw/excel/product_category_name_translation.xlsx
+++ b/data/raw/excel/product_category_name_translation.xlsx
@@ -8,15 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\brazilian-analytics\data\raw\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{105F6306-3DF8-4B76-8C37-0F65A82900A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9871003F-8F75-41B3-A68D-39DF15371B36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7860" yWindow="0" windowWidth="21045" windowHeight="15585" xr2:uid="{924CC56D-F169-4E2D-AF23-9C696523A0DB}"/>
+    <workbookView xWindow="7845" yWindow="0" windowWidth="21045" windowHeight="15585" activeTab="1" xr2:uid="{924CC56D-F169-4E2D-AF23-9C696523A0DB}"/>
   </bookViews>
   <sheets>
     <sheet name="product_category_name_translati" sheetId="1" r:id="rId1"/>
+    <sheet name="Category_Profile" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
       <xlwcv:version setVersion="1"/>
     </ext>
@@ -25,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="144">
   <si>
     <t>product_category_name</t>
   </si>
@@ -436,6 +448,27 @@
   </si>
   <si>
     <t>security_and_services</t>
+  </si>
+  <si>
+    <t>Check</t>
+  </si>
+  <si>
+    <t>Result</t>
+  </si>
+  <si>
+    <t>Number of Rows</t>
+  </si>
+  <si>
+    <t>Number of Columns</t>
+  </si>
+  <si>
+    <t>Missing Portuguese Category</t>
+  </si>
+  <si>
+    <t>Missing English Category</t>
+  </si>
+  <si>
+    <t>Duplicate Portuguese Categories</t>
   </si>
 </sst>
 </file>
@@ -979,6 +1012,17 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D9AEFA70-7FE6-44A7-AF9E-45AC4A26AFB0}" name="CategoryTranslation" displayName="CategoryTranslation" ref="A1:B72" totalsRowShown="0">
+  <autoFilter ref="A1:B72" xr:uid="{D9AEFA70-7FE6-44A7-AF9E-45AC4A26AFB0}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{DCC558DD-355A-4BD5-9187-31504CA1B1C9}" name="product_category_name"/>
+    <tableColumn id="2" xr3:uid="{A918BEC6-E09C-46E0-9AE9-F89DD468DFEB}" name="product_category_name_english"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1883,5 +1927,74 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7E45E3E4-A8D5-4B4D-A309-164974D9F583}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="30.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>139</v>
+      </c>
+      <c r="B2">
+        <f>ROWS(CategoryTranslation[])</f>
+        <v>71</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>140</v>
+      </c>
+      <c r="B3">
+        <f>COLUMNS(CategoryTranslation[#Headers])</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>141</v>
+      </c>
+      <c r="B4">
+        <f>COUNTBLANK(CategoryTranslation[product_category_name])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>142</v>
+      </c>
+      <c r="B5">
+        <f>COUNTBLANK(CategoryTranslation[product_category_name_english])</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>143</v>
+      </c>
+      <c r="B6">
+        <f>ROWS(CategoryTranslation[])-ROWS(_xlfn.UNIQUE(CategoryTranslation[product_category_name]))</f>
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>